<commit_message>
Enhance evaluation scripts and agent functionality
- Added a new evaluation command for running GAIA-style evaluations in `package.json`.
- Expanded the evaluation corpus with additional GAIA-style document QA cases, increasing the total to 67 cases.
- Improved the `run-full-eval` script to support forwarding additional arguments to the underlying `vitest` invocation.
- Enhanced diagnostics in the evaluation harness to capture stderr/stdout on failures, aiding in debugging.
- Updated tests to ensure reliability of new features and improved handling of evaluation cases.
</commit_message>
<xml_diff>
--- a/eval/fixtures/gaia/transactions.xlsx
+++ b/eval/fixtures/gaia/transactions.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -89,6 +89,15 @@
   </si>
   <si>
     <t>2024-03-22</t>
+  </si>
+  <si>
+    <t>2024-04-05</t>
+  </si>
+  <si>
+    <t>2024-04-15</t>
+  </si>
+  <si>
+    <t>2024-04-20</t>
   </si>
 </sst>
 </file>
@@ -465,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -656,6 +665,48 @@
         <v>16</v>
       </c>
     </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14">
+        <v>2000</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <v>3000</v>
+      </c>
+      <c r="D15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <v>1500</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>